<commit_message>
修复Excel场景覆盖列跨Method串联污染: PUT /api/Media、PUT /api/Media/complete、DELETE /api/CampaignTags三行标注纠正
update_excel.py的update_scenario_col在(method,path)精确匹配失败时会退化成"忽略method、按path合并所有case"，导致同路径不同method的行互相串场景文本(如PUT /api/Media错误显示了POST /api/Media创建流程的场景说明)。本地脚本已加method列存在时禁止跨method合并的判断(未提交，按规则脚本不入库)，本次手动核对并修正了受影响的3行数据。

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/single-api/walmart-api/swagger_modules.xlsx
+++ b/single-api/walmart-api/swagger_modules.xlsx
@@ -13992,11 +13992,9 @@
         </is>
       </c>
       <c r="E439" s="2" t="n"/>
-      <c r="F439" s="7" t="inlineStr">
-        <is>
-          <t>默认调用 — 99.4%
-创建标签→抓ID→删除(写操作·自清理)
-更新标签并绑定Campaign(写操作·自清理)</t>
+      <c r="F439" s="8" t="inlineStr">
+        <is>
+          <t>作为清理步骤(创建标签→抓ID→删除 / 更新标签并绑定Campaign 两条case内复用)</t>
         </is>
       </c>
       <c r="G439" s="4" t="inlineStr">
@@ -31557,10 +31555,9 @@
         </is>
       </c>
       <c r="E1104" s="2" t="n"/>
-      <c r="F1104" s="7" t="inlineStr">
-        <is>
-          <t>默认调用 — 100.0%
-上传视频素材(写操作·自清理，已用真实文件人工验证)</t>
+      <c r="F1104" s="8" t="inlineStr">
+        <is>
+          <t>默认调用 — 100.0%</t>
         </is>
       </c>
       <c r="G1104" s="4" t="inlineStr">
@@ -31788,7 +31785,7 @@
       <c r="E1112" s="2" t="n"/>
       <c r="F1112" s="8" t="inlineStr">
         <is>
-          <t>【仅生成未执行】完成媒体上传</t>
+          <t>上传视频素材(写操作·自清理，已用真实文件人工验证)</t>
         </is>
       </c>
       <c r="G1112" s="4" t="inlineStr">

</xml_diff>

<commit_message>
AdItems 2条ByCondition高危项处理完成: 限定测试账号campaign 426321+adGroup 770991122，2轮验证通过
按用户确认规则"只允许限定在自建测试实体"改造bid/byConditions与status/byConditions，
不再使用空条件数组(代表全账号范围)。两条均无配对还原步骤(ByCondition场景无GET原值接口)，
已在description注明。AdItems模块高危清单清理完毕。

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/single-api/walmart-api/swagger_modules.xlsx
+++ b/single-api/walmart-api/swagger_modules.xlsx
@@ -732,7 +732,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>86%(7执行,写操作4条未确认不计入)</t>
+          <t>73%</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -5669,7 +5669,7 @@
       <c r="E119" s="2" t="n"/>
       <c r="F119" s="7" t="inlineStr">
         <is>
-          <t>按条件批量改出价</t>
+          <t>按条件批量改出价(限定测试账号campaign+adGroup)</t>
         </is>
       </c>
       <c r="G119" s="4" t="inlineStr">
@@ -6098,7 +6098,7 @@
       <c r="E134" s="2" t="n"/>
       <c r="F134" s="7" t="inlineStr">
         <is>
-          <t>按条件批量改状态</t>
+          <t>按条件批量改状态(限定测试账号campaign+adGroup)</t>
         </is>
       </c>
       <c r="G134" s="4" t="inlineStr">

</xml_diff>